<commit_message>
Refitted model with UNAIDS 2025 data
- Biomodal fit in the Energy transition diagram - suggesting UNAIDS is diverging from other empirical data
- Proposing to reweight the data points for model fitting of the new UNAIDS data
</commit_message>
<xml_diff>
--- a/output/Chp2_tables/Chapter 2 - Table 1.xlsx
+++ b/output/Chp2_tables/Chapter 2 - Table 1.xlsx
@@ -184,85 +184,85 @@
     <t>0.13 to 2.06</t>
   </si>
   <si>
-    <t>14.3% (11.5% - 17.5%)</t>
+    <t>11.6% (9.4% - 14.7%)</t>
   </si>
   <si>
     <t>0.08 (0.03 - 0.16)</t>
   </si>
   <si>
-    <t>0.94 (0.45 - 1.88)</t>
-  </si>
-  <si>
-    <t>5.1% (4.2% - 6.2%)</t>
-  </si>
-  <si>
-    <t>1.6% (0.8% - 2.7%)</t>
-  </si>
-  <si>
-    <t>3.2% (1.8% - 5.3%)</t>
-  </si>
-  <si>
-    <t>0.25 (0.14 - 0.37)</t>
-  </si>
-  <si>
-    <t>0.35 (0.23 - 0.49)</t>
-  </si>
-  <si>
-    <t>81.7% (54.6% - 122.9%)</t>
-  </si>
-  <si>
-    <t>28.4% (17.7% - 49.3%)</t>
-  </si>
-  <si>
-    <t>48.6% (29.8% - 87.9%)</t>
-  </si>
-  <si>
-    <t>68.1% (29.0% - 135.5%)</t>
-  </si>
-  <si>
-    <t>10.3% (1.9% - 34.4%)</t>
-  </si>
-  <si>
-    <t>3.4% (2.0% - 5.3%)</t>
-  </si>
-  <si>
-    <t>2.2% (1.3% - 3.5%)</t>
-  </si>
-  <si>
-    <t>10.4% (5.5% - 18.6%)</t>
-  </si>
-  <si>
-    <t>7.5% (4.3% - 11.6%)</t>
-  </si>
-  <si>
-    <t>70.0% (41.9% - 91.1%)</t>
-  </si>
-  <si>
-    <t>21.5% (10.8% - 35.9%)</t>
-  </si>
-  <si>
-    <t>1.05 (0.73 - 1.55)</t>
-  </si>
-  <si>
-    <t>2.40 (1.49 - 3.55)</t>
-  </si>
-  <si>
-    <t>0.54 (0.18 - 1.25)</t>
-  </si>
-  <si>
-    <t>0.63 (0.34 - 1.07)</t>
-  </si>
-  <si>
-    <t>0.48 (0.24 - 0.84)</t>
-  </si>
-  <si>
-    <t>3.21 (1.60 - 5.86)</t>
-  </si>
-  <si>
-    <t>23.31 (20.10 - 25.89)</t>
-  </si>
-  <si>
-    <t>0.42 (0.11 - 1.13)</t>
+    <t>1.03 (0.62 - 2.37)</t>
+  </si>
+  <si>
+    <t>5.2% (4.4% - 6.1%)</t>
+  </si>
+  <si>
+    <t>1.7% (0.9% - 2.6%)</t>
+  </si>
+  <si>
+    <t>3.6% (2.5% - 5.9%)</t>
+  </si>
+  <si>
+    <t>0.28 (0.16 - 0.37)</t>
+  </si>
+  <si>
+    <t>0.32 (0.23 - 0.50)</t>
+  </si>
+  <si>
+    <t>88.8% (64.6% - 136.4%)</t>
+  </si>
+  <si>
+    <t>18.2% (11.6% - 35.3%)</t>
+  </si>
+  <si>
+    <t>46.9% (24.3% - 77.4%)</t>
+  </si>
+  <si>
+    <t>77.4% (37.3% - 132.0%)</t>
+  </si>
+  <si>
+    <t>14.3% (3.1% - 34.5%)</t>
+  </si>
+  <si>
+    <t>4.1% (2.3% - 5.6%)</t>
+  </si>
+  <si>
+    <t>2.0% (1.4% - 3.4%)</t>
+  </si>
+  <si>
+    <t>11.8% (6.1% - 20.0%)</t>
+  </si>
+  <si>
+    <t>6.9% (4.3% - 11.6%)</t>
+  </si>
+  <si>
+    <t>76.3% (42.4% - 89.7%)</t>
+  </si>
+  <si>
+    <t>20.8% (12.1% - 36.0%)</t>
+  </si>
+  <si>
+    <t>0.94 (0.72 - 1.48)</t>
+  </si>
+  <si>
+    <t>2.63 (1.57 - 3.47)</t>
+  </si>
+  <si>
+    <t>0.42 (0.13 - 1.25)</t>
+  </si>
+  <si>
+    <t>0.74 (0.36 - 1.04)</t>
+  </si>
+  <si>
+    <t>0.54 (0.22 - 0.81)</t>
+  </si>
+  <si>
+    <t>3.39 (1.62 - 5.64)</t>
+  </si>
+  <si>
+    <t>21.52 (20.15 - 25.77)</t>
+  </si>
+  <si>
+    <t>0.38 (0.14 - 1.29)</t>
   </si>
 </sst>
 </file>

</xml_diff>

<commit_message>
Revised model fittings - without changing weights/ Perfect fitting to UNAIDS
- Full rerun of Bayesian calibration, without changing the weights of the model
- This is the model fitting if UNAIDS modelling estimates are correct
- Perfect fitting to UNAIDS
</commit_message>
<xml_diff>
--- a/output/Chp2_tables/Chapter 2 - Table 1.xlsx
+++ b/output/Chp2_tables/Chapter 2 - Table 1.xlsx
@@ -184,85 +184,85 @@
     <t>0.13 to 2.06</t>
   </si>
   <si>
-    <t>11.6% (9.4% - 14.7%)</t>
+    <t>12.3% (9.5% - 15.2%)</t>
   </si>
   <si>
     <t>0.08 (0.03 - 0.16)</t>
   </si>
   <si>
-    <t>1.03 (0.62 - 2.37)</t>
-  </si>
-  <si>
-    <t>5.2% (4.4% - 6.1%)</t>
-  </si>
-  <si>
-    <t>1.7% (0.9% - 2.6%)</t>
-  </si>
-  <si>
-    <t>3.6% (2.5% - 5.9%)</t>
-  </si>
-  <si>
-    <t>0.28 (0.16 - 0.37)</t>
-  </si>
-  <si>
-    <t>0.32 (0.23 - 0.50)</t>
-  </si>
-  <si>
-    <t>88.8% (64.6% - 136.4%)</t>
-  </si>
-  <si>
-    <t>18.2% (11.6% - 35.3%)</t>
-  </si>
-  <si>
-    <t>46.9% (24.3% - 77.4%)</t>
-  </si>
-  <si>
-    <t>77.4% (37.3% - 132.0%)</t>
-  </si>
-  <si>
-    <t>14.3% (3.1% - 34.5%)</t>
-  </si>
-  <si>
-    <t>4.1% (2.3% - 5.6%)</t>
-  </si>
-  <si>
-    <t>2.0% (1.4% - 3.4%)</t>
-  </si>
-  <si>
-    <t>11.8% (6.1% - 20.0%)</t>
-  </si>
-  <si>
-    <t>6.9% (4.3% - 11.6%)</t>
-  </si>
-  <si>
-    <t>76.3% (42.4% - 89.7%)</t>
-  </si>
-  <si>
-    <t>20.8% (12.1% - 36.0%)</t>
-  </si>
-  <si>
-    <t>0.94 (0.72 - 1.48)</t>
-  </si>
-  <si>
-    <t>2.63 (1.57 - 3.47)</t>
-  </si>
-  <si>
-    <t>0.42 (0.13 - 1.25)</t>
-  </si>
-  <si>
-    <t>0.74 (0.36 - 1.04)</t>
-  </si>
-  <si>
-    <t>0.54 (0.22 - 0.81)</t>
-  </si>
-  <si>
-    <t>3.39 (1.62 - 5.64)</t>
-  </si>
-  <si>
-    <t>21.52 (20.15 - 25.77)</t>
-  </si>
-  <si>
-    <t>0.38 (0.14 - 1.29)</t>
+    <t>1.17 (0.61 - 2.40)</t>
+  </si>
+  <si>
+    <t>5.1% (4.3% - 6.1%)</t>
+  </si>
+  <si>
+    <t>1.7% (0.9% - 2.7%)</t>
+  </si>
+  <si>
+    <t>3.9% (2.3% - 6.0%)</t>
+  </si>
+  <si>
+    <t>0.25 (0.16 - 0.37)</t>
+  </si>
+  <si>
+    <t>0.36 (0.22 - 0.51)</t>
+  </si>
+  <si>
+    <t>93.7% (62.5% - 140.8%)</t>
+  </si>
+  <si>
+    <t>19.7% (12.6% - 35.1%)</t>
+  </si>
+  <si>
+    <t>43.3% (23.9% - 79.1%)</t>
+  </si>
+  <si>
+    <t>72.3% (32.6% - 133.4%)</t>
+  </si>
+  <si>
+    <t>11.3% (2.6% - 31.8%)</t>
+  </si>
+  <si>
+    <t>3.8% (2.3% - 5.7%)</t>
+  </si>
+  <si>
+    <t>2.2% (1.2% - 3.6%)</t>
+  </si>
+  <si>
+    <t>11.6% (6.4% - 21.7%)</t>
+  </si>
+  <si>
+    <t>7.5% (4.3% - 11.8%)</t>
+  </si>
+  <si>
+    <t>70.4% (41.3% - 90.3%)</t>
+  </si>
+  <si>
+    <t>21.7% (10.5% - 35.5%)</t>
+  </si>
+  <si>
+    <t>1.05 (0.71 - 1.50)</t>
+  </si>
+  <si>
+    <t>2.38 (1.53 - 3.62)</t>
+  </si>
+  <si>
+    <t>0.54 (0.18 - 1.16)</t>
+  </si>
+  <si>
+    <t>0.65 (0.35 - 1.11)</t>
+  </si>
+  <si>
+    <t>0.46 (0.22 - 0.87)</t>
+  </si>
+  <si>
+    <t>2.94 (1.56 - 5.57)</t>
+  </si>
+  <si>
+    <t>22.43 (20.11 - 25.85)</t>
+  </si>
+  <si>
+    <t>0.47 (0.12 - 1.27)</t>
   </si>
 </sst>
 </file>

</xml_diff>

<commit_message>
Another sets of weights to fit the model
- Not really reaching the historical data....
</commit_message>
<xml_diff>
--- a/output/Chp2_tables/Chapter 2 - Table 1.xlsx
+++ b/output/Chp2_tables/Chapter 2 - Table 1.xlsx
@@ -184,85 +184,85 @@
     <t>0.13 to 2.06</t>
   </si>
   <si>
-    <t>12.4% (9.7% - 15.4%)</t>
-  </si>
-  <si>
-    <t>0.08 (0.03 - 0.16)</t>
-  </si>
-  <si>
-    <t>1.22 (0.63 - 2.25)</t>
-  </si>
-  <si>
-    <t>5.1% (4.3% - 6.1%)</t>
-  </si>
-  <si>
-    <t>1.7% (0.9% - 2.7%)</t>
-  </si>
-  <si>
-    <t>4.0% (2.5% - 6.0%)</t>
-  </si>
-  <si>
-    <t>0.26 (0.16 - 0.38)</t>
-  </si>
-  <si>
-    <t>0.35 (0.23 - 0.51)</t>
-  </si>
-  <si>
-    <t>94.2% (61.5% - 136.4%)</t>
-  </si>
-  <si>
-    <t>20.4% (12.5% - 35.7%)</t>
-  </si>
-  <si>
-    <t>41.7% (23.5% - 80.2%)</t>
-  </si>
-  <si>
-    <t>72.9% (34.3% - 132.1%)</t>
-  </si>
-  <si>
-    <t>11.5% (2.8% - 35.5%)</t>
-  </si>
-  <si>
-    <t>3.7% (2.3% - 5.7%)</t>
-  </si>
-  <si>
-    <t>2.2% (1.3% - 3.6%)</t>
-  </si>
-  <si>
-    <t>11.7% (6.1% - 20.0%)</t>
-  </si>
-  <si>
-    <t>7.5% (4.5% - 11.6%)</t>
-  </si>
-  <si>
-    <t>70.7% (40.7% - 92.2%)</t>
-  </si>
-  <si>
-    <t>22.5% (11.6% - 35.4%)</t>
-  </si>
-  <si>
-    <t>1.03 (0.70 - 1.52)</t>
-  </si>
-  <si>
-    <t>2.37 (1.53 - 3.57)</t>
-  </si>
-  <si>
-    <t>0.54 (0.16 - 1.29)</t>
-  </si>
-  <si>
-    <t>0.66 (0.34 - 1.07)</t>
-  </si>
-  <si>
-    <t>0.46 (0.22 - 0.87)</t>
-  </si>
-  <si>
-    <t>2.80 (1.53 - 5.63)</t>
-  </si>
-  <si>
-    <t>22.48 (20.11 - 25.82)</t>
-  </si>
-  <si>
-    <t>0.47 (0.09 - 1.24)</t>
+    <t>11.9% (8.9% - 15.0%)</t>
+  </si>
+  <si>
+    <t>0.08 (0.03 - 0.17)</t>
+  </si>
+  <si>
+    <t>1.20 (0.61 - 2.38)</t>
+  </si>
+  <si>
+    <t>5.0% (4.2% - 6.1%)</t>
+  </si>
+  <si>
+    <t>1.6% (0.9% - 2.8%)</t>
+  </si>
+  <si>
+    <t>3.9% (2.4% - 6.3%)</t>
+  </si>
+  <si>
+    <t>0.25 (0.15 - 0.37)</t>
+  </si>
+  <si>
+    <t>0.36 (0.22 - 0.51)</t>
+  </si>
+  <si>
+    <t>95.3% (60.7% - 138.0%)</t>
+  </si>
+  <si>
+    <t>21.9% (13.4% - 37.4%)</t>
+  </si>
+  <si>
+    <t>41.6% (24.0% - 79.3%)</t>
+  </si>
+  <si>
+    <t>72.4% (36.4% - 132.8%)</t>
+  </si>
+  <si>
+    <t>10.9% (2.3% - 32.7%)</t>
+  </si>
+  <si>
+    <t>3.7% (2.2% - 5.6%)</t>
+  </si>
+  <si>
+    <t>2.2% (1.3% - 3.5%)</t>
+  </si>
+  <si>
+    <t>11.4% (6.3% - 20.9%)</t>
+  </si>
+  <si>
+    <t>7.5% (4.4% - 11.5%)</t>
+  </si>
+  <si>
+    <t>70.7% (41.1% - 89.9%)</t>
+  </si>
+  <si>
+    <t>21.8% (11.3% - 35.7%)</t>
+  </si>
+  <si>
+    <t>1.04 (0.69 - 1.48)</t>
+  </si>
+  <si>
+    <t>2.39 (1.46 - 3.47)</t>
+  </si>
+  <si>
+    <t>0.54 (0.20 - 1.18)</t>
+  </si>
+  <si>
+    <t>0.63 (0.35 - 1.11)</t>
+  </si>
+  <si>
+    <t>0.45 (0.22 - 0.86)</t>
+  </si>
+  <si>
+    <t>3.03 (1.56 - 5.70)</t>
+  </si>
+  <si>
+    <t>22.32 (20.10 - 25.74)</t>
+  </si>
+  <si>
+    <t>0.63 (0.20 - 1.36)</t>
   </si>
 </sst>
 </file>

</xml_diff>

<commit_message>
Recalibrate by pulling more weights to historical data
- More pulling to the historical data
</commit_message>
<xml_diff>
--- a/output/Chp2_tables/Chapter 2 - Table 1.xlsx
+++ b/output/Chp2_tables/Chapter 2 - Table 1.xlsx
@@ -184,85 +184,85 @@
     <t>0.13 to 2.06</t>
   </si>
   <si>
-    <t>11.9% (8.9% - 15.0%)</t>
-  </si>
-  <si>
-    <t>0.08 (0.03 - 0.17)</t>
-  </si>
-  <si>
-    <t>1.20 (0.61 - 2.38)</t>
-  </si>
-  <si>
-    <t>5.0% (4.2% - 6.1%)</t>
-  </si>
-  <si>
-    <t>1.6% (0.9% - 2.8%)</t>
-  </si>
-  <si>
-    <t>3.9% (2.4% - 6.3%)</t>
+    <t>12.0% (9.1% - 14.9%)</t>
+  </si>
+  <si>
+    <t>0.08 (0.03 - 0.16)</t>
+  </si>
+  <si>
+    <t>1.20 (0.60 - 2.39)</t>
+  </si>
+  <si>
+    <t>5.1% (4.2% - 6.2%)</t>
+  </si>
+  <si>
+    <t>1.6% (0.8% - 2.8%)</t>
+  </si>
+  <si>
+    <t>4.2% (2.5% - 6.4%)</t>
   </si>
   <si>
     <t>0.25 (0.15 - 0.37)</t>
   </si>
   <si>
-    <t>0.36 (0.22 - 0.51)</t>
-  </si>
-  <si>
-    <t>95.3% (60.7% - 138.0%)</t>
-  </si>
-  <si>
-    <t>21.9% (13.4% - 37.4%)</t>
-  </si>
-  <si>
-    <t>41.6% (24.0% - 79.3%)</t>
-  </si>
-  <si>
-    <t>72.4% (36.4% - 132.8%)</t>
-  </si>
-  <si>
-    <t>10.9% (2.3% - 32.7%)</t>
-  </si>
-  <si>
-    <t>3.7% (2.2% - 5.6%)</t>
+    <t>0.35 (0.23 - 0.49)</t>
+  </si>
+  <si>
+    <t>93.5% (61.9% - 139.7%)</t>
+  </si>
+  <si>
+    <t>22.5% (13.9% - 40.7%)</t>
+  </si>
+  <si>
+    <t>40.8% (23.9% - 73.7%)</t>
+  </si>
+  <si>
+    <t>72.6% (35.0% - 132.6%)</t>
+  </si>
+  <si>
+    <t>11.4% (2.2% - 35.2%)</t>
+  </si>
+  <si>
+    <t>3.7% (2.2% - 5.7%)</t>
   </si>
   <si>
     <t>2.2% (1.3% - 3.5%)</t>
   </si>
   <si>
-    <t>11.4% (6.3% - 20.9%)</t>
-  </si>
-  <si>
-    <t>7.5% (4.4% - 11.5%)</t>
-  </si>
-  <si>
-    <t>70.7% (41.1% - 89.9%)</t>
-  </si>
-  <si>
-    <t>21.8% (11.3% - 35.7%)</t>
-  </si>
-  <si>
-    <t>1.04 (0.69 - 1.48)</t>
-  </si>
-  <si>
-    <t>2.39 (1.46 - 3.47)</t>
-  </si>
-  <si>
-    <t>0.54 (0.20 - 1.18)</t>
-  </si>
-  <si>
-    <t>0.63 (0.35 - 1.11)</t>
-  </si>
-  <si>
-    <t>0.45 (0.22 - 0.86)</t>
-  </si>
-  <si>
-    <t>3.03 (1.56 - 5.70)</t>
-  </si>
-  <si>
-    <t>22.32 (20.10 - 25.74)</t>
-  </si>
-  <si>
-    <t>0.63 (0.20 - 1.36)</t>
+    <t>11.6% (6.1% - 20.3%)</t>
+  </si>
+  <si>
+    <t>7.5% (4.3% - 12.0%)</t>
+  </si>
+  <si>
+    <t>71.0% (41.1% - 90.3%)</t>
+  </si>
+  <si>
+    <t>22.4% (11.3% - 35.1%)</t>
+  </si>
+  <si>
+    <t>1.05 (0.69 - 1.56)</t>
+  </si>
+  <si>
+    <t>2.39 (1.47 - 3.51)</t>
+  </si>
+  <si>
+    <t>0.55 (0.19 - 1.25)</t>
+  </si>
+  <si>
+    <t>0.64 (0.34 - 1.09)</t>
+  </si>
+  <si>
+    <t>0.45 (0.22 - 0.83)</t>
+  </si>
+  <si>
+    <t>3.06 (1.56 - 5.70)</t>
+  </si>
+  <si>
+    <t>22.39 (20.08 - 25.78)</t>
+  </si>
+  <si>
+    <t>0.61 (0.18 - 1.35)</t>
   </si>
 </sst>
 </file>

</xml_diff>

<commit_message>
Covering entirety of historical data
- New recalibration to cover all historical data and pass through UNAIDS estimates
</commit_message>
<xml_diff>
--- a/output/Chp2_tables/Chapter 2 - Table 1.xlsx
+++ b/output/Chp2_tables/Chapter 2 - Table 1.xlsx
@@ -184,85 +184,85 @@
     <t>0.13 to 2.06</t>
   </si>
   <si>
-    <t>12.0% (9.1% - 14.9%)</t>
-  </si>
-  <si>
-    <t>0.08 (0.03 - 0.16)</t>
-  </si>
-  <si>
-    <t>1.20 (0.60 - 2.39)</t>
-  </si>
-  <si>
-    <t>5.1% (4.2% - 6.2%)</t>
-  </si>
-  <si>
-    <t>1.6% (0.8% - 2.8%)</t>
-  </si>
-  <si>
-    <t>4.2% (2.5% - 6.4%)</t>
-  </si>
-  <si>
-    <t>0.25 (0.15 - 0.37)</t>
-  </si>
-  <si>
-    <t>0.35 (0.23 - 0.49)</t>
-  </si>
-  <si>
-    <t>93.5% (61.9% - 139.7%)</t>
-  </si>
-  <si>
-    <t>22.5% (13.9% - 40.7%)</t>
-  </si>
-  <si>
-    <t>40.8% (23.9% - 73.7%)</t>
-  </si>
-  <si>
-    <t>72.6% (35.0% - 132.6%)</t>
-  </si>
-  <si>
-    <t>11.4% (2.2% - 35.2%)</t>
-  </si>
-  <si>
-    <t>3.7% (2.2% - 5.7%)</t>
+    <t>12.1% (8.4% - 16.6%)</t>
+  </si>
+  <si>
+    <t>0.08 (0.03 - 0.17)</t>
+  </si>
+  <si>
+    <t>0.97 (0.42 - 2.16)</t>
+  </si>
+  <si>
+    <t>5.2% (4.2% - 6.5%)</t>
+  </si>
+  <si>
+    <t>1.8% (0.9% - 3.1%)</t>
+  </si>
+  <si>
+    <t>4.7% (2.4% - 8.1%)</t>
+  </si>
+  <si>
+    <t>0.26 (0.16 - 0.38)</t>
+  </si>
+  <si>
+    <t>0.36 (0.22 - 0.51)</t>
+  </si>
+  <si>
+    <t>85.3% (54.7% - 131.5%)</t>
+  </si>
+  <si>
+    <t>21.6% (9.6% - 45.5%)</t>
+  </si>
+  <si>
+    <t>45.9% (19.9% - 93.3%)</t>
+  </si>
+  <si>
+    <t>68.9% (32.0% - 128.1%)</t>
+  </si>
+  <si>
+    <t>10.7% (2.9% - 31.0%)</t>
+  </si>
+  <si>
+    <t>3.4% (2.0% - 5.3%)</t>
   </si>
   <si>
     <t>2.2% (1.3% - 3.5%)</t>
   </si>
   <si>
-    <t>11.6% (6.1% - 20.3%)</t>
-  </si>
-  <si>
-    <t>7.5% (4.3% - 12.0%)</t>
-  </si>
-  <si>
-    <t>71.0% (41.1% - 90.3%)</t>
-  </si>
-  <si>
-    <t>22.4% (11.3% - 35.1%)</t>
-  </si>
-  <si>
-    <t>1.05 (0.69 - 1.56)</t>
-  </si>
-  <si>
-    <t>2.39 (1.47 - 3.51)</t>
-  </si>
-  <si>
-    <t>0.55 (0.19 - 1.25)</t>
-  </si>
-  <si>
-    <t>0.64 (0.34 - 1.09)</t>
-  </si>
-  <si>
-    <t>0.45 (0.22 - 0.83)</t>
-  </si>
-  <si>
-    <t>3.06 (1.56 - 5.70)</t>
-  </si>
-  <si>
-    <t>22.39 (20.08 - 25.78)</t>
-  </si>
-  <si>
-    <t>0.61 (0.18 - 1.35)</t>
+    <t>10.7% (5.6% - 19.4%)</t>
+  </si>
+  <si>
+    <t>7.6% (4.4% - 11.7%)</t>
+  </si>
+  <si>
+    <t>69.6% (41.7% - 91.5%)</t>
+  </si>
+  <si>
+    <t>22.1% (12.5% - 34.7%)</t>
+  </si>
+  <si>
+    <t>1.04 (0.70 - 1.50)</t>
+  </si>
+  <si>
+    <t>2.40 (1.48 - 3.73)</t>
+  </si>
+  <si>
+    <t>0.59 (0.19 - 1.33)</t>
+  </si>
+  <si>
+    <t>0.65 (0.34 - 1.08)</t>
+  </si>
+  <si>
+    <t>0.49 (0.22 - 0.90)</t>
+  </si>
+  <si>
+    <t>3.38 (1.59 - 5.84)</t>
+  </si>
+  <si>
+    <t>22.97 (20.11 - 25.86)</t>
+  </si>
+  <si>
+    <t>0.67 (0.12 - 1.89)</t>
   </si>
 </sst>
 </file>

</xml_diff>

<commit_message>
Another fittings to cover historical data
- Another set of refits with different weights
</commit_message>
<xml_diff>
--- a/output/Chp2_tables/Chapter 2 - Table 1.xlsx
+++ b/output/Chp2_tables/Chapter 2 - Table 1.xlsx
@@ -184,85 +184,85 @@
     <t>0.13 to 2.06</t>
   </si>
   <si>
-    <t>12.1% (8.4% - 16.6%)</t>
+    <t>12.2% (8.8% - 16.1%)</t>
   </si>
   <si>
     <t>0.08 (0.03 - 0.17)</t>
   </si>
   <si>
-    <t>0.97 (0.42 - 2.16)</t>
-  </si>
-  <si>
-    <t>5.2% (4.2% - 6.5%)</t>
-  </si>
-  <si>
-    <t>1.8% (0.9% - 3.1%)</t>
-  </si>
-  <si>
-    <t>4.7% (2.4% - 8.1%)</t>
+    <t>0.98 (0.43 - 2.16)</t>
+  </si>
+  <si>
+    <t>5.2% (4.3% - 6.5%)</t>
+  </si>
+  <si>
+    <t>1.8% (0.9% - 3.0%)</t>
+  </si>
+  <si>
+    <t>4.7% (2.4% - 8.2%)</t>
   </si>
   <si>
     <t>0.26 (0.16 - 0.38)</t>
   </si>
   <si>
-    <t>0.36 (0.22 - 0.51)</t>
-  </si>
-  <si>
-    <t>85.3% (54.7% - 131.5%)</t>
-  </si>
-  <si>
-    <t>21.6% (9.6% - 45.5%)</t>
-  </si>
-  <si>
-    <t>45.9% (19.9% - 93.3%)</t>
-  </si>
-  <si>
-    <t>68.9% (32.0% - 128.1%)</t>
-  </si>
-  <si>
-    <t>10.7% (2.9% - 31.0%)</t>
-  </si>
-  <si>
-    <t>3.4% (2.0% - 5.3%)</t>
-  </si>
-  <si>
-    <t>2.2% (1.3% - 3.5%)</t>
-  </si>
-  <si>
-    <t>10.7% (5.6% - 19.4%)</t>
-  </si>
-  <si>
-    <t>7.6% (4.4% - 11.7%)</t>
-  </si>
-  <si>
-    <t>69.6% (41.7% - 91.5%)</t>
-  </si>
-  <si>
-    <t>22.1% (12.5% - 34.7%)</t>
-  </si>
-  <si>
-    <t>1.04 (0.70 - 1.50)</t>
-  </si>
-  <si>
-    <t>2.40 (1.48 - 3.73)</t>
-  </si>
-  <si>
-    <t>0.59 (0.19 - 1.33)</t>
-  </si>
-  <si>
-    <t>0.65 (0.34 - 1.08)</t>
-  </si>
-  <si>
-    <t>0.49 (0.22 - 0.90)</t>
-  </si>
-  <si>
-    <t>3.38 (1.59 - 5.84)</t>
-  </si>
-  <si>
-    <t>22.97 (20.11 - 25.86)</t>
-  </si>
-  <si>
-    <t>0.67 (0.12 - 1.89)</t>
+    <t>0.35 (0.23 - 0.50)</t>
+  </si>
+  <si>
+    <t>86.8% (52.9% - 141.8%)</t>
+  </si>
+  <si>
+    <t>20.8% (9.5% - 43.4%)</t>
+  </si>
+  <si>
+    <t>45.5% (21.0% - 93.8%)</t>
+  </si>
+  <si>
+    <t>68.9% (32.6% - 124.2%)</t>
+  </si>
+  <si>
+    <t>10.6% (2.8% - 29.6%)</t>
+  </si>
+  <si>
+    <t>3.5% (2.1% - 5.5%)</t>
+  </si>
+  <si>
+    <t>2.2% (1.3% - 3.4%)</t>
+  </si>
+  <si>
+    <t>10.8% (5.8% - 19.3%)</t>
+  </si>
+  <si>
+    <t>7.5% (4.1% - 12.2%)</t>
+  </si>
+  <si>
+    <t>70.2% (41.3% - 90.2%)</t>
+  </si>
+  <si>
+    <t>21.9% (12.1% - 34.7%)</t>
+  </si>
+  <si>
+    <t>1.03 (0.71 - 1.58)</t>
+  </si>
+  <si>
+    <t>2.34 (1.48 - 3.59)</t>
+  </si>
+  <si>
+    <t>0.57 (0.20 - 1.25)</t>
+  </si>
+  <si>
+    <t>0.64 (0.33 - 1.12)</t>
+  </si>
+  <si>
+    <t>0.49 (0.23 - 0.94)</t>
+  </si>
+  <si>
+    <t>3.35 (1.60 - 5.84)</t>
+  </si>
+  <si>
+    <t>22.93 (20.13 - 25.86)</t>
+  </si>
+  <si>
+    <t>0.68 (0.13 - 1.73)</t>
   </si>
 </sst>
 </file>

</xml_diff>

<commit_message>
New recalibration that follows new UNAIDS estimates
- recalibrate again to UNAIDS
</commit_message>
<xml_diff>
--- a/output/Chp2_tables/Chapter 2 - Table 1.xlsx
+++ b/output/Chp2_tables/Chapter 2 - Table 1.xlsx
@@ -184,85 +184,85 @@
     <t>0.13 to 2.06</t>
   </si>
   <si>
-    <t>12.2% (8.8% - 16.1%)</t>
-  </si>
-  <si>
-    <t>0.08 (0.03 - 0.17)</t>
-  </si>
-  <si>
-    <t>0.98 (0.43 - 2.16)</t>
-  </si>
-  <si>
-    <t>5.2% (4.3% - 6.5%)</t>
-  </si>
-  <si>
-    <t>1.8% (0.9% - 3.0%)</t>
-  </si>
-  <si>
-    <t>4.7% (2.4% - 8.2%)</t>
-  </si>
-  <si>
-    <t>0.26 (0.16 - 0.38)</t>
-  </si>
-  <si>
-    <t>0.35 (0.23 - 0.50)</t>
-  </si>
-  <si>
-    <t>86.8% (52.9% - 141.8%)</t>
-  </si>
-  <si>
-    <t>20.8% (9.5% - 43.4%)</t>
-  </si>
-  <si>
-    <t>45.5% (21.0% - 93.8%)</t>
-  </si>
-  <si>
-    <t>68.9% (32.6% - 124.2%)</t>
-  </si>
-  <si>
-    <t>10.6% (2.8% - 29.6%)</t>
-  </si>
-  <si>
-    <t>3.5% (2.1% - 5.5%)</t>
-  </si>
-  <si>
-    <t>2.2% (1.3% - 3.4%)</t>
-  </si>
-  <si>
-    <t>10.8% (5.8% - 19.3%)</t>
-  </si>
-  <si>
-    <t>7.5% (4.1% - 12.2%)</t>
-  </si>
-  <si>
-    <t>70.2% (41.3% - 90.2%)</t>
-  </si>
-  <si>
-    <t>21.9% (12.1% - 34.7%)</t>
-  </si>
-  <si>
-    <t>1.03 (0.71 - 1.58)</t>
-  </si>
-  <si>
-    <t>2.34 (1.48 - 3.59)</t>
-  </si>
-  <si>
-    <t>0.57 (0.20 - 1.25)</t>
-  </si>
-  <si>
-    <t>0.64 (0.33 - 1.12)</t>
-  </si>
-  <si>
-    <t>0.49 (0.23 - 0.94)</t>
-  </si>
-  <si>
-    <t>3.35 (1.60 - 5.84)</t>
-  </si>
-  <si>
-    <t>22.93 (20.13 - 25.86)</t>
-  </si>
-  <si>
-    <t>0.68 (0.13 - 1.73)</t>
+    <t>12.1% (9.5% - 14.9%)</t>
+  </si>
+  <si>
+    <t>0.08 (0.03 - 0.18)</t>
+  </si>
+  <si>
+    <t>1.18 (0.59 - 2.30)</t>
+  </si>
+  <si>
+    <t>5.0% (4.3% - 6.1%)</t>
+  </si>
+  <si>
+    <t>1.6% (0.9% - 2.7%)</t>
+  </si>
+  <si>
+    <t>3.8% (2.3% - 5.8%)</t>
+  </si>
+  <si>
+    <t>0.25 (0.15 - 0.38)</t>
+  </si>
+  <si>
+    <t>0.36 (0.22 - 0.52)</t>
+  </si>
+  <si>
+    <t>95.6% (62.8% - 142.7%)</t>
+  </si>
+  <si>
+    <t>19.9% (12.7% - 35.3%)</t>
+  </si>
+  <si>
+    <t>41.0% (23.8% - 75.9%)</t>
+  </si>
+  <si>
+    <t>74.2% (35.7% - 129.7%)</t>
+  </si>
+  <si>
+    <t>11.5% (2.5% - 34.8%)</t>
+  </si>
+  <si>
+    <t>3.8% (2.4% - 5.6%)</t>
+  </si>
+  <si>
+    <t>2.2% (1.3% - 3.5%)</t>
+  </si>
+  <si>
+    <t>11.8% (6.4% - 20.9%)</t>
+  </si>
+  <si>
+    <t>7.5% (4.5% - 11.6%)</t>
+  </si>
+  <si>
+    <t>69.4% (39.2% - 90.3%)</t>
+  </si>
+  <si>
+    <t>22.2% (12.4% - 36.0%)</t>
+  </si>
+  <si>
+    <t>1.03 (0.71 - 1.48)</t>
+  </si>
+  <si>
+    <t>2.36 (1.49 - 3.57)</t>
+  </si>
+  <si>
+    <t>0.54 (0.18 - 1.15)</t>
+  </si>
+  <si>
+    <t>0.65 (0.36 - 1.15)</t>
+  </si>
+  <si>
+    <t>0.46 (0.20 - 0.86)</t>
+  </si>
+  <si>
+    <t>3.00 (1.58 - 5.60)</t>
+  </si>
+  <si>
+    <t>22.46 (20.10 - 25.69)</t>
+  </si>
+  <si>
+    <t>0.49 (0.11 - 1.30)</t>
   </si>
 </sst>
 </file>

</xml_diff>

<commit_message>
different set of weights to pull the empirical data closer
- not really closer?
</commit_message>
<xml_diff>
--- a/output/Chp2_tables/Chapter 2 - Table 1.xlsx
+++ b/output/Chp2_tables/Chapter 2 - Table 1.xlsx
@@ -184,85 +184,85 @@
     <t>0.13 to 2.06</t>
   </si>
   <si>
-    <t>12.1% (9.5% - 14.9%)</t>
-  </si>
-  <si>
-    <t>0.08 (0.03 - 0.18)</t>
-  </si>
-  <si>
-    <t>1.18 (0.59 - 2.30)</t>
-  </si>
-  <si>
-    <t>5.0% (4.3% - 6.1%)</t>
-  </si>
-  <si>
-    <t>1.6% (0.9% - 2.7%)</t>
-  </si>
-  <si>
-    <t>3.8% (2.3% - 5.8%)</t>
-  </si>
-  <si>
-    <t>0.25 (0.15 - 0.38)</t>
-  </si>
-  <si>
-    <t>0.36 (0.22 - 0.52)</t>
-  </si>
-  <si>
-    <t>95.6% (62.8% - 142.7%)</t>
-  </si>
-  <si>
-    <t>19.9% (12.7% - 35.3%)</t>
-  </si>
-  <si>
-    <t>41.0% (23.8% - 75.9%)</t>
-  </si>
-  <si>
-    <t>74.2% (35.7% - 129.7%)</t>
-  </si>
-  <si>
-    <t>11.5% (2.5% - 34.8%)</t>
-  </si>
-  <si>
-    <t>3.8% (2.4% - 5.6%)</t>
-  </si>
-  <si>
-    <t>2.2% (1.3% - 3.5%)</t>
-  </si>
-  <si>
-    <t>11.8% (6.4% - 20.9%)</t>
-  </si>
-  <si>
-    <t>7.5% (4.5% - 11.6%)</t>
-  </si>
-  <si>
-    <t>69.4% (39.2% - 90.3%)</t>
-  </si>
-  <si>
-    <t>22.2% (12.4% - 36.0%)</t>
-  </si>
-  <si>
-    <t>1.03 (0.71 - 1.48)</t>
-  </si>
-  <si>
-    <t>2.36 (1.49 - 3.57)</t>
-  </si>
-  <si>
-    <t>0.54 (0.18 - 1.15)</t>
-  </si>
-  <si>
-    <t>0.65 (0.36 - 1.15)</t>
-  </si>
-  <si>
-    <t>0.46 (0.20 - 0.86)</t>
-  </si>
-  <si>
-    <t>3.00 (1.58 - 5.60)</t>
-  </si>
-  <si>
-    <t>22.46 (20.10 - 25.69)</t>
-  </si>
-  <si>
-    <t>0.49 (0.11 - 1.30)</t>
+    <t>11.9% (8.2% - 16.1%)</t>
+  </si>
+  <si>
+    <t>0.08 (0.03 - 0.16)</t>
+  </si>
+  <si>
+    <t>0.96 (0.47 - 2.19)</t>
+  </si>
+  <si>
+    <t>5.2% (4.3% - 6.5%)</t>
+  </si>
+  <si>
+    <t>1.8% (1.0% - 3.1%)</t>
+  </si>
+  <si>
+    <t>4.7% (2.4% - 7.9%)</t>
+  </si>
+  <si>
+    <t>0.26 (0.16 - 0.38)</t>
+  </si>
+  <si>
+    <t>0.36 (0.22 - 0.51)</t>
+  </si>
+  <si>
+    <t>85.9% (52.0% - 135.8%)</t>
+  </si>
+  <si>
+    <t>21.4% (9.2% - 45.8%)</t>
+  </si>
+  <si>
+    <t>45.9% (20.8% - 90.1%)</t>
+  </si>
+  <si>
+    <t>71.3% (31.5% - 131.6%)</t>
+  </si>
+  <si>
+    <t>10.6% (2.1% - 32.4%)</t>
+  </si>
+  <si>
+    <t>3.4% (2.0% - 5.4%)</t>
+  </si>
+  <si>
+    <t>2.3% (1.2% - 3.5%)</t>
+  </si>
+  <si>
+    <t>10.8% (5.4% - 19.6%)</t>
+  </si>
+  <si>
+    <t>7.6% (4.5% - 11.3%)</t>
+  </si>
+  <si>
+    <t>69.8% (40.3% - 90.2%)</t>
+  </si>
+  <si>
+    <t>21.9% (12.2% - 34.1%)</t>
+  </si>
+  <si>
+    <t>1.04 (0.67 - 1.60)</t>
+  </si>
+  <si>
+    <t>2.37 (1.48 - 3.47)</t>
+  </si>
+  <si>
+    <t>0.57 (0.19 - 1.26)</t>
+  </si>
+  <si>
+    <t>0.64 (0.35 - 1.11)</t>
+  </si>
+  <si>
+    <t>0.48 (0.23 - 0.93)</t>
+  </si>
+  <si>
+    <t>3.51 (1.57 - 5.88)</t>
+  </si>
+  <si>
+    <t>23.03 (20.16 - 25.87)</t>
+  </si>
+  <si>
+    <t>0.66 (0.14 - 1.77)</t>
   </si>
 </sst>
 </file>

</xml_diff>

<commit_message>
Heavy weights on the historical data recalibration
- Recalibration on historical data
</commit_message>
<xml_diff>
--- a/output/Chp2_tables/Chapter 2 - Table 1.xlsx
+++ b/output/Chp2_tables/Chapter 2 - Table 1.xlsx
@@ -184,85 +184,85 @@
     <t>0.13 to 2.06</t>
   </si>
   <si>
-    <t>11.9% (8.2% - 16.1%)</t>
+    <t>11.8% (9.0% - 14.7%)</t>
   </si>
   <si>
     <t>0.08 (0.03 - 0.16)</t>
   </si>
   <si>
-    <t>0.96 (0.47 - 2.19)</t>
-  </si>
-  <si>
-    <t>5.2% (4.3% - 6.5%)</t>
-  </si>
-  <si>
-    <t>1.8% (1.0% - 3.1%)</t>
-  </si>
-  <si>
-    <t>4.7% (2.4% - 7.9%)</t>
-  </si>
-  <si>
-    <t>0.26 (0.16 - 0.38)</t>
-  </si>
-  <si>
-    <t>0.36 (0.22 - 0.51)</t>
-  </si>
-  <si>
-    <t>85.9% (52.0% - 135.8%)</t>
-  </si>
-  <si>
-    <t>21.4% (9.2% - 45.8%)</t>
-  </si>
-  <si>
-    <t>45.9% (20.8% - 90.1%)</t>
-  </si>
-  <si>
-    <t>71.3% (31.5% - 131.6%)</t>
-  </si>
-  <si>
-    <t>10.6% (2.1% - 32.4%)</t>
-  </si>
-  <si>
-    <t>3.4% (2.0% - 5.4%)</t>
-  </si>
-  <si>
-    <t>2.3% (1.2% - 3.5%)</t>
-  </si>
-  <si>
-    <t>10.8% (5.4% - 19.6%)</t>
-  </si>
-  <si>
-    <t>7.6% (4.5% - 11.3%)</t>
-  </si>
-  <si>
-    <t>69.8% (40.3% - 90.2%)</t>
-  </si>
-  <si>
-    <t>21.9% (12.2% - 34.1%)</t>
-  </si>
-  <si>
-    <t>1.04 (0.67 - 1.60)</t>
-  </si>
-  <si>
-    <t>2.37 (1.48 - 3.47)</t>
-  </si>
-  <si>
-    <t>0.57 (0.19 - 1.26)</t>
-  </si>
-  <si>
-    <t>0.64 (0.35 - 1.11)</t>
-  </si>
-  <si>
-    <t>0.48 (0.23 - 0.93)</t>
-  </si>
-  <si>
-    <t>3.51 (1.57 - 5.88)</t>
-  </si>
-  <si>
-    <t>23.03 (20.16 - 25.87)</t>
-  </si>
-  <si>
-    <t>0.66 (0.14 - 1.77)</t>
+    <t>1.20 (0.63 - 2.46)</t>
+  </si>
+  <si>
+    <t>5.0% (4.2% - 6.1%)</t>
+  </si>
+  <si>
+    <t>1.6% (0.8% - 2.7%)</t>
+  </si>
+  <si>
+    <t>4.1% (2.5% - 6.2%)</t>
+  </si>
+  <si>
+    <t>0.25 (0.15 - 0.37)</t>
+  </si>
+  <si>
+    <t>0.35 (0.22 - 0.51)</t>
+  </si>
+  <si>
+    <t>94.5% (63.1% - 139.2%)</t>
+  </si>
+  <si>
+    <t>22.4% (13.9% - 41.1%)</t>
+  </si>
+  <si>
+    <t>41.8% (23.9% - 79.6%)</t>
+  </si>
+  <si>
+    <t>73.4% (36.9% - 127.1%)</t>
+  </si>
+  <si>
+    <t>11.1% (2.3% - 32.3%)</t>
+  </si>
+  <si>
+    <t>3.7% (2.2% - 5.6%)</t>
+  </si>
+  <si>
+    <t>2.2% (1.2% - 3.5%)</t>
+  </si>
+  <si>
+    <t>11.6% (6.1% - 19.8%)</t>
+  </si>
+  <si>
+    <t>7.6% (4.6% - 11.6%)</t>
+  </si>
+  <si>
+    <t>69.9% (39.0% - 90.5%)</t>
+  </si>
+  <si>
+    <t>22.1% (12.6% - 36.1%)</t>
+  </si>
+  <si>
+    <t>1.04 (0.70 - 1.57)</t>
+  </si>
+  <si>
+    <t>2.36 (1.49 - 3.63)</t>
+  </si>
+  <si>
+    <t>0.56 (0.18 - 1.27)</t>
+  </si>
+  <si>
+    <t>0.65 (0.35 - 1.11)</t>
+  </si>
+  <si>
+    <t>0.45 (0.22 - 0.80)</t>
+  </si>
+  <si>
+    <t>3.09 (1.56 - 5.77)</t>
+  </si>
+  <si>
+    <t>22.32 (20.12 - 25.56)</t>
+  </si>
+  <si>
+    <t>0.63 (0.20 - 1.33)</t>
   </si>
 </sst>
 </file>

</xml_diff>

<commit_message>
Update the year when diagnoses ramp up - recalibrate
- UNAIDS is suggesting a later trends of diagnoses
</commit_message>
<xml_diff>
--- a/output/Chp2_tables/Chapter 2 - Table 1.xlsx
+++ b/output/Chp2_tables/Chapter 2 - Table 1.xlsx
@@ -184,85 +184,85 @@
     <t>0.13 to 2.06</t>
   </si>
   <si>
-    <t>11.8% (9.0% - 14.7%)</t>
+    <t>12.0% (9.2% - 14.8%)</t>
   </si>
   <si>
     <t>0.08 (0.03 - 0.16)</t>
   </si>
   <si>
-    <t>1.20 (0.63 - 2.46)</t>
-  </si>
-  <si>
-    <t>5.0% (4.2% - 6.1%)</t>
-  </si>
-  <si>
-    <t>1.6% (0.8% - 2.7%)</t>
-  </si>
-  <si>
-    <t>4.1% (2.5% - 6.2%)</t>
-  </si>
-  <si>
-    <t>0.25 (0.15 - 0.37)</t>
+    <t>1.28 (0.64 - 2.55)</t>
+  </si>
+  <si>
+    <t>5.1% (4.2% - 6.3%)</t>
+  </si>
+  <si>
+    <t>1.7% (0.8% - 2.9%)</t>
+  </si>
+  <si>
+    <t>4.2% (2.6% - 6.1%)</t>
+  </si>
+  <si>
+    <t>0.25 (0.15 - 0.39)</t>
   </si>
   <si>
     <t>0.35 (0.22 - 0.51)</t>
   </si>
   <si>
-    <t>94.5% (63.1% - 139.2%)</t>
-  </si>
-  <si>
-    <t>22.4% (13.9% - 41.1%)</t>
-  </si>
-  <si>
-    <t>41.8% (23.9% - 79.6%)</t>
-  </si>
-  <si>
-    <t>73.4% (36.9% - 127.1%)</t>
-  </si>
-  <si>
-    <t>11.1% (2.3% - 32.3%)</t>
-  </si>
-  <si>
-    <t>3.7% (2.2% - 5.6%)</t>
-  </si>
-  <si>
-    <t>2.2% (1.2% - 3.5%)</t>
-  </si>
-  <si>
-    <t>11.6% (6.1% - 19.8%)</t>
-  </si>
-  <si>
-    <t>7.6% (4.6% - 11.6%)</t>
-  </si>
-  <si>
-    <t>69.9% (39.0% - 90.5%)</t>
-  </si>
-  <si>
-    <t>22.1% (12.6% - 36.1%)</t>
-  </si>
-  <si>
-    <t>1.04 (0.70 - 1.57)</t>
-  </si>
-  <si>
-    <t>2.36 (1.49 - 3.63)</t>
-  </si>
-  <si>
-    <t>0.56 (0.18 - 1.27)</t>
-  </si>
-  <si>
-    <t>0.65 (0.35 - 1.11)</t>
-  </si>
-  <si>
-    <t>0.45 (0.22 - 0.80)</t>
-  </si>
-  <si>
-    <t>3.09 (1.56 - 5.77)</t>
-  </si>
-  <si>
-    <t>22.32 (20.12 - 25.56)</t>
-  </si>
-  <si>
-    <t>0.63 (0.20 - 1.33)</t>
+    <t>97.8% (64.8% - 146.2%)</t>
+  </si>
+  <si>
+    <t>20.3% (13.4% - 34.4%)</t>
+  </si>
+  <si>
+    <t>55.5% (31.4% - 101.4%)</t>
+  </si>
+  <si>
+    <t>74.7% (36.1% - 138.8%)</t>
+  </si>
+  <si>
+    <t>11.8% (2.8% - 32.7%)</t>
+  </si>
+  <si>
+    <t>3.8% (2.4% - 5.8%)</t>
+  </si>
+  <si>
+    <t>2.2% (1.3% - 3.5%)</t>
+  </si>
+  <si>
+    <t>11.9% (6.5% - 21.0%)</t>
+  </si>
+  <si>
+    <t>7.5% (4.5% - 12.1%)</t>
+  </si>
+  <si>
+    <t>69.6% (38.6% - 90.4%)</t>
+  </si>
+  <si>
+    <t>21.3% (10.7% - 34.6%)</t>
+  </si>
+  <si>
+    <t>1.03 (0.71 - 1.52)</t>
+  </si>
+  <si>
+    <t>2.36 (1.48 - 3.56)</t>
+  </si>
+  <si>
+    <t>0.55 (0.21 - 1.23)</t>
+  </si>
+  <si>
+    <t>0.61 (0.32 - 1.11)</t>
+  </si>
+  <si>
+    <t>0.54 (0.28 - 0.93)</t>
+  </si>
+  <si>
+    <t>2.97 (1.57 - 5.70)</t>
+  </si>
+  <si>
+    <t>22.59 (20.17 - 25.61)</t>
+  </si>
+  <si>
+    <t>0.62 (0.15 - 1.47)</t>
   </si>
 </sst>
 </file>

</xml_diff>

<commit_message>
Revise the weights of treatments
</commit_message>
<xml_diff>
--- a/output/Chp2_tables/Chapter 2 - Table 1.xlsx
+++ b/output/Chp2_tables/Chapter 2 - Table 1.xlsx
@@ -184,85 +184,85 @@
     <t>0.13 to 2.06</t>
   </si>
   <si>
-    <t>12.0% (9.2% - 14.8%)</t>
-  </si>
-  <si>
-    <t>0.08 (0.03 - 0.16)</t>
-  </si>
-  <si>
-    <t>1.28 (0.64 - 2.55)</t>
-  </si>
-  <si>
-    <t>5.1% (4.2% - 6.3%)</t>
-  </si>
-  <si>
-    <t>1.7% (0.8% - 2.9%)</t>
-  </si>
-  <si>
-    <t>4.2% (2.6% - 6.1%)</t>
-  </si>
-  <si>
-    <t>0.25 (0.15 - 0.39)</t>
-  </si>
-  <si>
-    <t>0.35 (0.22 - 0.51)</t>
-  </si>
-  <si>
-    <t>97.8% (64.8% - 146.2%)</t>
-  </si>
-  <si>
-    <t>20.3% (13.4% - 34.4%)</t>
-  </si>
-  <si>
-    <t>55.5% (31.4% - 101.4%)</t>
-  </si>
-  <si>
-    <t>74.7% (36.1% - 138.8%)</t>
-  </si>
-  <si>
-    <t>11.8% (2.8% - 32.7%)</t>
-  </si>
-  <si>
-    <t>3.8% (2.4% - 5.8%)</t>
-  </si>
-  <si>
-    <t>2.2% (1.3% - 3.5%)</t>
-  </si>
-  <si>
-    <t>11.9% (6.5% - 21.0%)</t>
-  </si>
-  <si>
-    <t>7.5% (4.5% - 12.1%)</t>
-  </si>
-  <si>
-    <t>69.6% (38.6% - 90.4%)</t>
-  </si>
-  <si>
-    <t>21.3% (10.7% - 34.6%)</t>
-  </si>
-  <si>
-    <t>1.03 (0.71 - 1.52)</t>
-  </si>
-  <si>
-    <t>2.36 (1.48 - 3.56)</t>
-  </si>
-  <si>
-    <t>0.55 (0.21 - 1.23)</t>
-  </si>
-  <si>
-    <t>0.61 (0.32 - 1.11)</t>
-  </si>
-  <si>
-    <t>0.54 (0.28 - 0.93)</t>
-  </si>
-  <si>
-    <t>2.97 (1.57 - 5.70)</t>
-  </si>
-  <si>
-    <t>22.59 (20.17 - 25.61)</t>
-  </si>
-  <si>
-    <t>0.62 (0.15 - 1.47)</t>
+    <t>11.9% (9.4% - 14.9%)</t>
+  </si>
+  <si>
+    <t>0.08 (0.03 - 0.17)</t>
+  </si>
+  <si>
+    <t>1.31 (0.63 - 2.66)</t>
+  </si>
+  <si>
+    <t>5.1% (4.3% - 6.3%)</t>
+  </si>
+  <si>
+    <t>1.7% (0.9% - 2.9%)</t>
+  </si>
+  <si>
+    <t>4.1% (2.5% - 6.3%)</t>
+  </si>
+  <si>
+    <t>0.25 (0.16 - 0.37)</t>
+  </si>
+  <si>
+    <t>0.35 (0.23 - 0.50)</t>
+  </si>
+  <si>
+    <t>97.1% (63.7% - 145.6%)</t>
+  </si>
+  <si>
+    <t>20.6% (13.2% - 34.8%)</t>
+  </si>
+  <si>
+    <t>56.6% (31.5% - 106.1%)</t>
+  </si>
+  <si>
+    <t>76.8% (37.1% - 135.8%)</t>
+  </si>
+  <si>
+    <t>11.6% (2.7% - 34.7%)</t>
+  </si>
+  <si>
+    <t>3.8% (2.3% - 5.8%)</t>
+  </si>
+  <si>
+    <t>2.2% (1.2% - 3.5%)</t>
+  </si>
+  <si>
+    <t>11.8% (6.4% - 21.2%)</t>
+  </si>
+  <si>
+    <t>7.5% (4.4% - 12.3%)</t>
+  </si>
+  <si>
+    <t>70.1% (40.6% - 90.2%)</t>
+  </si>
+  <si>
+    <t>21.6% (11.1% - 34.8%)</t>
+  </si>
+  <si>
+    <t>1.03 (0.69 - 1.57)</t>
+  </si>
+  <si>
+    <t>2.38 (1.49 - 3.49)</t>
+  </si>
+  <si>
+    <t>0.56 (0.20 - 1.20)</t>
+  </si>
+  <si>
+    <t>0.59 (0.31 - 1.05)</t>
+  </si>
+  <si>
+    <t>0.53 (0.27 - 0.94)</t>
+  </si>
+  <si>
+    <t>2.96 (1.56 - 5.76)</t>
+  </si>
+  <si>
+    <t>22.41 (20.13 - 25.74)</t>
+  </si>
+  <si>
+    <t>0.62 (0.18 - 1.51)</t>
   </si>
 </sst>
 </file>

</xml_diff>

<commit_message>
Revised the weights of treatment initiations and diagnoses in the model
- Trying to match new UNAIDS treatment and diagnoses (superficial issues)
</commit_message>
<xml_diff>
--- a/output/Chp2_tables/Chapter 2 - Table 1.xlsx
+++ b/output/Chp2_tables/Chapter 2 - Table 1.xlsx
@@ -184,13 +184,13 @@
     <t>0.13 to 2.06</t>
   </si>
   <si>
-    <t>11.9% (9.4% - 14.9%)</t>
+    <t>12.0% (9.2% - 14.9%)</t>
   </si>
   <si>
     <t>0.08 (0.03 - 0.17)</t>
   </si>
   <si>
-    <t>1.31 (0.63 - 2.66)</t>
+    <t>1.21 (0.64 - 2.29)</t>
   </si>
   <si>
     <t>5.1% (4.3% - 6.3%)</t>
@@ -199,70 +199,70 @@
     <t>1.7% (0.9% - 2.9%)</t>
   </si>
   <si>
-    <t>4.1% (2.5% - 6.3%)</t>
+    <t>4.0% (2.4% - 6.2%)</t>
   </si>
   <si>
     <t>0.25 (0.16 - 0.37)</t>
   </si>
   <si>
-    <t>0.35 (0.23 - 0.50)</t>
-  </si>
-  <si>
-    <t>97.1% (63.7% - 145.6%)</t>
-  </si>
-  <si>
-    <t>20.6% (13.2% - 34.8%)</t>
-  </si>
-  <si>
-    <t>56.6% (31.5% - 106.1%)</t>
-  </si>
-  <si>
-    <t>76.8% (37.1% - 135.8%)</t>
-  </si>
-  <si>
-    <t>11.6% (2.7% - 34.7%)</t>
-  </si>
-  <si>
-    <t>3.8% (2.3% - 5.8%)</t>
-  </si>
-  <si>
-    <t>2.2% (1.2% - 3.5%)</t>
-  </si>
-  <si>
-    <t>11.8% (6.4% - 21.2%)</t>
-  </si>
-  <si>
-    <t>7.5% (4.4% - 12.3%)</t>
-  </si>
-  <si>
-    <t>70.1% (40.6% - 90.2%)</t>
-  </si>
-  <si>
-    <t>21.6% (11.1% - 34.8%)</t>
-  </si>
-  <si>
-    <t>1.03 (0.69 - 1.57)</t>
-  </si>
-  <si>
-    <t>2.38 (1.49 - 3.49)</t>
-  </si>
-  <si>
-    <t>0.56 (0.20 - 1.20)</t>
-  </si>
-  <si>
-    <t>0.59 (0.31 - 1.05)</t>
-  </si>
-  <si>
-    <t>0.53 (0.27 - 0.94)</t>
-  </si>
-  <si>
-    <t>2.96 (1.56 - 5.76)</t>
-  </si>
-  <si>
-    <t>22.41 (20.13 - 25.74)</t>
-  </si>
-  <si>
-    <t>0.62 (0.18 - 1.51)</t>
+    <t>0.35 (0.22 - 0.50)</t>
+  </si>
+  <si>
+    <t>95.4% (62.2% - 146.8%)</t>
+  </si>
+  <si>
+    <t>17.2% (10.5% - 31.6%)</t>
+  </si>
+  <si>
+    <t>48.9% (26.7% - 91.2%)</t>
+  </si>
+  <si>
+    <t>71.3% (36.7% - 130.1%)</t>
+  </si>
+  <si>
+    <t>11.0% (2.5% - 31.3%)</t>
+  </si>
+  <si>
+    <t>3.7% (2.2% - 5.6%)</t>
+  </si>
+  <si>
+    <t>2.2% (1.3% - 3.5%)</t>
+  </si>
+  <si>
+    <t>11.6% (5.8% - 21.3%)</t>
+  </si>
+  <si>
+    <t>7.6% (4.5% - 11.7%)</t>
+  </si>
+  <si>
+    <t>70.1% (42.1% - 90.2%)</t>
+  </si>
+  <si>
+    <t>21.6% (11.2% - 34.6%)</t>
+  </si>
+  <si>
+    <t>1.04 (0.70 - 1.60)</t>
+  </si>
+  <si>
+    <t>2.35 (1.45 - 3.55)</t>
+  </si>
+  <si>
+    <t>0.55 (0.18 - 1.28)</t>
+  </si>
+  <si>
+    <t>0.63 (0.34 - 1.08)</t>
+  </si>
+  <si>
+    <t>0.47 (0.22 - 0.88)</t>
+  </si>
+  <si>
+    <t>2.88 (1.54 - 5.85)</t>
+  </si>
+  <si>
+    <t>22.50 (20.12 - 25.70)</t>
+  </si>
+  <si>
+    <t>0.55 (0.11 - 1.40)</t>
   </si>
 </sst>
 </file>

</xml_diff>

<commit_message>
Revise weights in the model for treatment (again)
</commit_message>
<xml_diff>
--- a/output/Chp2_tables/Chapter 2 - Table 1.xlsx
+++ b/output/Chp2_tables/Chapter 2 - Table 1.xlsx
@@ -184,85 +184,85 @@
     <t>0.13 to 2.06</t>
   </si>
   <si>
-    <t>12.0% (9.2% - 14.9%)</t>
-  </si>
-  <si>
-    <t>0.08 (0.03 - 0.17)</t>
-  </si>
-  <si>
-    <t>1.21 (0.64 - 2.29)</t>
-  </si>
-  <si>
-    <t>5.1% (4.3% - 6.3%)</t>
-  </si>
-  <si>
-    <t>1.7% (0.9% - 2.9%)</t>
-  </si>
-  <si>
-    <t>4.0% (2.4% - 6.2%)</t>
-  </si>
-  <si>
-    <t>0.25 (0.16 - 0.37)</t>
-  </si>
-  <si>
-    <t>0.35 (0.22 - 0.50)</t>
-  </si>
-  <si>
-    <t>95.4% (62.2% - 146.8%)</t>
-  </si>
-  <si>
-    <t>17.2% (10.5% - 31.6%)</t>
-  </si>
-  <si>
-    <t>48.9% (26.7% - 91.2%)</t>
-  </si>
-  <si>
-    <t>71.3% (36.7% - 130.1%)</t>
-  </si>
-  <si>
-    <t>11.0% (2.5% - 31.3%)</t>
-  </si>
-  <si>
-    <t>3.7% (2.2% - 5.6%)</t>
-  </si>
-  <si>
-    <t>2.2% (1.3% - 3.5%)</t>
-  </si>
-  <si>
-    <t>11.6% (5.8% - 21.3%)</t>
-  </si>
-  <si>
-    <t>7.6% (4.5% - 11.7%)</t>
-  </si>
-  <si>
-    <t>70.1% (42.1% - 90.2%)</t>
-  </si>
-  <si>
-    <t>21.6% (11.2% - 34.6%)</t>
-  </si>
-  <si>
-    <t>1.04 (0.70 - 1.60)</t>
-  </si>
-  <si>
-    <t>2.35 (1.45 - 3.55)</t>
-  </si>
-  <si>
-    <t>0.55 (0.18 - 1.28)</t>
-  </si>
-  <si>
-    <t>0.63 (0.34 - 1.08)</t>
-  </si>
-  <si>
-    <t>0.47 (0.22 - 0.88)</t>
-  </si>
-  <si>
-    <t>2.88 (1.54 - 5.85)</t>
-  </si>
-  <si>
-    <t>22.50 (20.12 - 25.70)</t>
-  </si>
-  <si>
-    <t>0.55 (0.11 - 1.40)</t>
+    <t>12.0% (9.2% - 15.1%)</t>
+  </si>
+  <si>
+    <t>0.08 (0.03 - 0.16)</t>
+  </si>
+  <si>
+    <t>1.20 (0.60 - 2.42)</t>
+  </si>
+  <si>
+    <t>5.1% (4.3% - 6.2%)</t>
+  </si>
+  <si>
+    <t>1.7% (0.9% - 2.8%)</t>
+  </si>
+  <si>
+    <t>4.0% (2.4% - 6.1%)</t>
+  </si>
+  <si>
+    <t>0.25 (0.15 - 0.38)</t>
+  </si>
+  <si>
+    <t>0.35 (0.21 - 0.50)</t>
+  </si>
+  <si>
+    <t>93.8% (59.6% - 141.3%)</t>
+  </si>
+  <si>
+    <t>17.5% (10.9% - 33.2%)</t>
+  </si>
+  <si>
+    <t>48.7% (27.0% - 84.6%)</t>
+  </si>
+  <si>
+    <t>73.6% (37.3% - 135.1%)</t>
+  </si>
+  <si>
+    <t>11.4% (2.8% - 35.2%)</t>
+  </si>
+  <si>
+    <t>3.7% (2.3% - 5.7%)</t>
+  </si>
+  <si>
+    <t>2.2% (1.3% - 3.4%)</t>
+  </si>
+  <si>
+    <t>11.8% (5.8% - 20.4%)</t>
+  </si>
+  <si>
+    <t>7.5% (4.3% - 11.6%)</t>
+  </si>
+  <si>
+    <t>69.6% (41.0% - 90.1%)</t>
+  </si>
+  <si>
+    <t>21.6% (11.6% - 34.5%)</t>
+  </si>
+  <si>
+    <t>1.05 (0.69 - 1.55)</t>
+  </si>
+  <si>
+    <t>2.38 (1.52 - 3.49)</t>
+  </si>
+  <si>
+    <t>0.54 (0.17 - 1.20)</t>
+  </si>
+  <si>
+    <t>0.64 (0.34 - 1.14)</t>
+  </si>
+  <si>
+    <t>0.47 (0.23 - 0.86)</t>
+  </si>
+  <si>
+    <t>2.99 (1.56 - 5.78)</t>
+  </si>
+  <si>
+    <t>22.40 (20.10 - 25.82)</t>
+  </si>
+  <si>
+    <t>0.53 (0.14 - 1.34)</t>
   </si>
 </sst>
 </file>

</xml_diff>

<commit_message>
Remove weights on the historical prevalence
- no longer consider historical prevalence data (which were UNAIDS-sourced) in the calibration
</commit_message>
<xml_diff>
--- a/output/Chp2_tables/Chapter 2 - Table 1.xlsx
+++ b/output/Chp2_tables/Chapter 2 - Table 1.xlsx
@@ -184,85 +184,85 @@
     <t>0.13 to 2.06</t>
   </si>
   <si>
-    <t>12.0% (9.2% - 15.1%)</t>
-  </si>
-  <si>
-    <t>0.08 (0.03 - 0.16)</t>
-  </si>
-  <si>
-    <t>1.20 (0.60 - 2.42)</t>
-  </si>
-  <si>
-    <t>5.1% (4.3% - 6.2%)</t>
+    <t>12.0% (9.2% - 15.0%)</t>
+  </si>
+  <si>
+    <t>0.08 (0.03 - 0.17)</t>
+  </si>
+  <si>
+    <t>1.21 (0.59 - 2.33)</t>
+  </si>
+  <si>
+    <t>5.1% (4.2% - 6.2%)</t>
   </si>
   <si>
     <t>1.7% (0.9% - 2.8%)</t>
   </si>
   <si>
-    <t>4.0% (2.4% - 6.1%)</t>
-  </si>
-  <si>
-    <t>0.25 (0.15 - 0.38)</t>
-  </si>
-  <si>
-    <t>0.35 (0.21 - 0.50)</t>
-  </si>
-  <si>
-    <t>93.8% (59.6% - 141.3%)</t>
-  </si>
-  <si>
-    <t>17.5% (10.9% - 33.2%)</t>
-  </si>
-  <si>
-    <t>48.7% (27.0% - 84.6%)</t>
-  </si>
-  <si>
-    <t>73.6% (37.3% - 135.1%)</t>
-  </si>
-  <si>
-    <t>11.4% (2.8% - 35.2%)</t>
-  </si>
-  <si>
-    <t>3.7% (2.3% - 5.7%)</t>
-  </si>
-  <si>
-    <t>2.2% (1.3% - 3.4%)</t>
-  </si>
-  <si>
-    <t>11.8% (5.8% - 20.4%)</t>
-  </si>
-  <si>
-    <t>7.5% (4.3% - 11.6%)</t>
-  </si>
-  <si>
-    <t>69.6% (41.0% - 90.1%)</t>
-  </si>
-  <si>
-    <t>21.6% (11.6% - 34.5%)</t>
-  </si>
-  <si>
-    <t>1.05 (0.69 - 1.55)</t>
-  </si>
-  <si>
-    <t>2.38 (1.52 - 3.49)</t>
-  </si>
-  <si>
-    <t>0.54 (0.17 - 1.20)</t>
-  </si>
-  <si>
-    <t>0.64 (0.34 - 1.14)</t>
-  </si>
-  <si>
-    <t>0.47 (0.23 - 0.86)</t>
-  </si>
-  <si>
-    <t>2.99 (1.56 - 5.78)</t>
-  </si>
-  <si>
-    <t>22.40 (20.10 - 25.82)</t>
-  </si>
-  <si>
-    <t>0.53 (0.14 - 1.34)</t>
+    <t>4.0% (2.5% - 6.1%)</t>
+  </si>
+  <si>
+    <t>0.25 (0.16 - 0.37)</t>
+  </si>
+  <si>
+    <t>0.35 (0.22 - 0.50)</t>
+  </si>
+  <si>
+    <t>96.9% (63.0% - 141.6%)</t>
+  </si>
+  <si>
+    <t>17.6% (11.0% - 32.4%)</t>
+  </si>
+  <si>
+    <t>48.6% (26.8% - 86.1%)</t>
+  </si>
+  <si>
+    <t>73.1% (34.3% - 134.7%)</t>
+  </si>
+  <si>
+    <t>11.4% (2.3% - 37.2%)</t>
+  </si>
+  <si>
+    <t>3.7% (2.3% - 5.6%)</t>
+  </si>
+  <si>
+    <t>2.2% (1.3% - 3.5%)</t>
+  </si>
+  <si>
+    <t>11.3% (6.3% - 19.8%)</t>
+  </si>
+  <si>
+    <t>7.6% (4.3% - 11.8%)</t>
+  </si>
+  <si>
+    <t>69.9% (39.5% - 90.1%)</t>
+  </si>
+  <si>
+    <t>21.8% (11.5% - 35.5%)</t>
+  </si>
+  <si>
+    <t>1.05 (0.71 - 1.58)</t>
+  </si>
+  <si>
+    <t>2.39 (1.48 - 3.64)</t>
+  </si>
+  <si>
+    <t>0.54 (0.17 - 1.24)</t>
+  </si>
+  <si>
+    <t>0.64 (0.32 - 1.11)</t>
+  </si>
+  <si>
+    <t>0.46 (0.24 - 0.85)</t>
+  </si>
+  <si>
+    <t>3.00 (1.56 - 5.72)</t>
+  </si>
+  <si>
+    <t>22.61 (20.14 - 25.86)</t>
+  </si>
+  <si>
+    <t>0.53 (0.13 - 1.31)</t>
   </si>
 </sst>
 </file>

</xml_diff>